<commit_message>
Updated BNC connector info
</commit_message>
<xml_diff>
--- a/PCB/V2/CAMOutputs/CL02_V2_BOM.xlsx
+++ b/PCB/V2/CAMOutputs/CL02_V2_BOM.xlsx
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="114">
   <si>
     <t>Qty</t>
   </si>
@@ -387,16 +387,27 @@
   </si>
   <si>
     <t>*DNP=Do not place</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/Superbat-Connector-Bulkhead-Monitoring-Transceiver/dp/B09V56M8F4/ref=sxin_17_pa_sp_search_thematic_sspa?content-id=amzn1.sym.141f5c48-2844-433f-b731-f8ecc97a5095%3Aamzn1.sym.141f5c48-2844-433f-b731-f8ecc97a5095&amp;crid=2UQMM3WBVRV0B&amp;cv_ct_cx=bnc%2Bconnector%2Bboard&amp;keywords=bnc%2Bconnector%2Bboard&amp;pd_rd_i=B09V56M8F4&amp;pd_rd_r=bcac4005-43c4-4c71-a401-e3c8c18935dd&amp;pd_rd_w=Pdc8j&amp;pd_rd_wg=vB4hv&amp;pf_rd_p=141f5c48-2844-433f-b731-f8ecc97a5095&amp;pf_rd_r=71A9AARRTYG4VHMEDEJM&amp;qid=1774940759&amp;sbo=RZvfv%2F%2FHxDF%2BO5021pAnSA%3D%3D&amp;sprefix=bnc%2Bconnector%2Bboar%2Caps%2C204&amp;sr=1-1-6024b2a3-78e4-4fed-8fed-e1613be3bcce-spons&amp;aref=gE7PPDgKRK&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9zZWFyY2hfdGhlbWF0aWM&amp;th=1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -425,14 +436,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1085,8 +1099,8 @@
       <c r="E14" t="s">
         <v>55</v>
       </c>
-      <c r="F14" t="s">
-        <v>99</v>
+      <c r="F14" s="2" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.3">

</xml_diff>